<commit_message>
Align instrument ranges with installation register
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D3 Physical rationality and rate constraints/outputs/data/D3_physical_events.xlsx
+++ b/Project 1 Data Quality Assessment/D3 Physical rationality and rate constraints/outputs/data/D3_physical_events.xlsx
@@ -214,10 +214,10 @@
     <t>rate_violation</t>
   </si>
   <si>
-    <t>instrument_range</t>
-  </si>
-  <si>
-    <t>hard_violation;instrument_range</t>
+    <t>hard_bound</t>
+  </si>
+  <si>
+    <t>hard_violation</t>
   </si>
   <si>
     <t>medium</t>
@@ -226,7 +226,7 @@
     <t>high</t>
   </si>
   <si>
-    <t>RUN_D3_v2.2.0_20260726T084811Z_4246fb53</t>
+    <t>RUN_D3_v2.2.1_20260727T043759Z_8d52c551</t>
   </si>
 </sst>
 </file>
@@ -719,7 +719,7 @@
         <v>120</v>
       </c>
       <c r="G4">
-        <v>1.5</v>
+        <v>1.900110579605932</v>
       </c>
       <c r="H4" t="b">
         <v>1</v>
@@ -1422,7 +1422,7 @@
         <v>120</v>
       </c>
       <c r="G24">
-        <v>1.5</v>
+        <v>1.900573785227608</v>
       </c>
       <c r="H24" t="b">
         <v>1</v>
@@ -1495,7 +1495,7 @@
         <v>120</v>
       </c>
       <c r="G26">
-        <v>1.5</v>
+        <v>1.76689093150976</v>
       </c>
       <c r="H26" t="b">
         <v>1</v>
@@ -1533,7 +1533,7 @@
         <v>120</v>
       </c>
       <c r="G27">
-        <v>1.5</v>
+        <v>1.900001006115465</v>
       </c>
       <c r="H27" t="b">
         <v>1</v>
@@ -1571,7 +1571,7 @@
         <v>120</v>
       </c>
       <c r="G28">
-        <v>1.5</v>
+        <v>1.900001006115465</v>
       </c>
       <c r="H28" t="b">
         <v>1</v>
@@ -1609,7 +1609,7 @@
         <v>120</v>
       </c>
       <c r="G29">
-        <v>1.5</v>
+        <v>1.900001006115465</v>
       </c>
       <c r="H29" t="b">
         <v>1</v>
@@ -1647,7 +1647,7 @@
         <v>120</v>
       </c>
       <c r="G30">
-        <v>1.5</v>
+        <v>1.900001006115465</v>
       </c>
       <c r="H30" t="b">
         <v>1</v>
@@ -1685,7 +1685,7 @@
         <v>120</v>
       </c>
       <c r="G31">
-        <v>1.5</v>
+        <v>1.900001006115465</v>
       </c>
       <c r="H31" t="b">
         <v>1</v>
@@ -1723,7 +1723,7 @@
         <v>120</v>
       </c>
       <c r="G32">
-        <v>1.5</v>
+        <v>1.900001006115465</v>
       </c>
       <c r="H32" t="b">
         <v>1</v>
@@ -1761,7 +1761,7 @@
         <v>120</v>
       </c>
       <c r="G33">
-        <v>1.5</v>
+        <v>1.900001006115465</v>
       </c>
       <c r="H33" t="b">
         <v>1</v>
@@ -1799,7 +1799,7 @@
         <v>120</v>
       </c>
       <c r="G34">
-        <v>1.5</v>
+        <v>1.900001007657574</v>
       </c>
       <c r="H34" t="b">
         <v>1</v>
@@ -1837,7 +1837,7 @@
         <v>120</v>
       </c>
       <c r="G35">
-        <v>1.5</v>
+        <v>1.900003979247734</v>
       </c>
       <c r="H35" t="b">
         <v>1</v>
@@ -1875,7 +1875,7 @@
         <v>120</v>
       </c>
       <c r="G36">
-        <v>1.5</v>
+        <v>1.900001006115465</v>
       </c>
       <c r="H36" t="b">
         <v>1</v>
@@ -1913,7 +1913,7 @@
         <v>120</v>
       </c>
       <c r="G37">
-        <v>1.5</v>
+        <v>1.900001006115465</v>
       </c>
       <c r="H37" t="b">
         <v>1</v>
@@ -1951,7 +1951,7 @@
         <v>120</v>
       </c>
       <c r="G38">
-        <v>1.5</v>
+        <v>1.900001006115465</v>
       </c>
       <c r="H38" t="b">
         <v>1</v>
@@ -1989,7 +1989,7 @@
         <v>120</v>
       </c>
       <c r="G39">
-        <v>1.5</v>
+        <v>1.900001006115465</v>
       </c>
       <c r="H39" t="b">
         <v>1</v>
@@ -2027,7 +2027,7 @@
         <v>120</v>
       </c>
       <c r="G40">
-        <v>1.5</v>
+        <v>1.900002413540903</v>
       </c>
       <c r="H40" t="b">
         <v>1</v>
@@ -2065,7 +2065,7 @@
         <v>120</v>
       </c>
       <c r="G41">
-        <v>1.5</v>
+        <v>1.900001006115465</v>
       </c>
       <c r="H41" t="b">
         <v>1</v>
@@ -2103,7 +2103,7 @@
         <v>120</v>
       </c>
       <c r="G42">
-        <v>1.5</v>
+        <v>1.900001006115465</v>
       </c>
       <c r="H42" t="b">
         <v>1</v>
@@ -2141,7 +2141,7 @@
         <v>120</v>
       </c>
       <c r="G43">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="H43" t="b">
         <v>1</v>
@@ -2153,7 +2153,7 @@
         <v>0</v>
       </c>
       <c r="K43" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L43" t="s">
         <v>70</v>
@@ -2179,7 +2179,7 @@
         <v>120</v>
       </c>
       <c r="G44">
-        <v>1.5</v>
+        <v>1.900001006115465</v>
       </c>
       <c r="H44" t="b">
         <v>1</v>
@@ -2217,7 +2217,7 @@
         <v>120</v>
       </c>
       <c r="G45">
-        <v>1.5</v>
+        <v>1.900001006115465</v>
       </c>
       <c r="H45" t="b">
         <v>1</v>
@@ -2255,7 +2255,7 @@
         <v>120</v>
       </c>
       <c r="G46">
-        <v>1.5</v>
+        <v>1.900001006115465</v>
       </c>
       <c r="H46" t="b">
         <v>1</v>
@@ -2293,7 +2293,7 @@
         <v>120</v>
       </c>
       <c r="G47">
-        <v>1.5</v>
+        <v>1.900002217861359</v>
       </c>
       <c r="H47" t="b">
         <v>1</v>
@@ -2366,7 +2366,7 @@
         <v>120</v>
       </c>
       <c r="G49">
-        <v>1.5</v>
+        <v>1.900023063063201</v>
       </c>
       <c r="H49" t="b">
         <v>1</v>
@@ -2404,7 +2404,7 @@
         <v>120</v>
       </c>
       <c r="G50">
-        <v>1.5</v>
+        <v>1.900001006125856</v>
       </c>
       <c r="H50" t="b">
         <v>1</v>
@@ -2442,7 +2442,7 @@
         <v>120</v>
       </c>
       <c r="G51">
-        <v>1.5</v>
+        <v>1.900001234984781</v>
       </c>
       <c r="H51" t="b">
         <v>1</v>

</xml_diff>